<commit_message>
Fix Product 5.0 improvement limits
</commit_message>
<xml_diff>
--- a/distribution/SIMS-Blog-Manager-template-Product5.0-Official.xlsx
+++ b/distribution/SIMS-Blog-Manager-template-Product5.0-Official.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="Raf192664648248c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R421c430acac149c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="Ra1b380221cb0481f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R41b3b4c89c344f97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="効果測定" sheetId="5" r:id="R43f8851cdaee40bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="R70b7a09df5e94936"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="R65c60dfbec46470e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="Rbac0cb5773264f3e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R198b101e833540ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R94a4e7aeb1144d83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R2f4a7c6b8d684b45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R8816b06011ce4700"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R78f8822310f64223"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="Rdae8a45d47aa41ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R7e323f17811547c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="効果測定" sheetId="5" r:id="Re3dd538dc9c14521"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Rc301332d438d4951"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="Rf1554d820878463a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R490f0cb56ae04a74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R3592beb284ec42c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="Rcc2568e64c4c4bd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="Rb96b150dec8f4b9e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -470,7 +470,7 @@
         <x:v>バージョン</x:v>
       </x:c>
       <x:c r="B2" s="33" t="str">
-        <x:v>4.3.0-rc1</x:v>
+        <x:v>5.0.0-official</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -9412,7 +9412,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B2" s="28" t="str">
-        <x:v>4.3.0-rc1</x:v>
+        <x:v>5.0.0-official</x:v>
       </x:c>
       <x:c r="C2" s="28" t="str">
         <x:v>システムバージョン</x:v>
@@ -9526,94 +9526,130 @@
         <x:v>QueueLimit</x:v>
       </x:c>
       <x:c r="B12" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>今日の改善に表示する件数。通常は5件</x:v>
+        <x:v>今日の改善の初期表示件数</x:v>
       </x:c>
       <x:c r="D12" t="str"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>TodayDisplayMode</x:v>
-      </x:c>
-      <x:c r="B13" t="str">
-        <x:v>TOP5</x:v>
+        <x:v>TodayInitialDisplayCount</x:v>
+      </x:c>
+      <x:c r="B13" t="n">
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C13" t="str">
-        <x:v>TOP5またはALL</x:v>
-      </x:c>
-      <x:c r="D13" t="str"/>
+        <x:v>今日の改善の初期表示件数</x:v>
+      </x:c>
+      <x:c r="D13"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>RelatedQueries</x:v>
+        <x:v>TodayMaxDisplayCount</x:v>
       </x:c>
       <x:c r="B14" t="n">
-        <x:v>20</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>改善ブリーフ用クエリ件数</x:v>
-      </x:c>
-      <x:c r="D14" t="str"/>
+        <x:v>今日の改善の最大表示件数</x:v>
+      </x:c>
+      <x:c r="D14"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
-        <x:v>MinImpressions</x:v>
+        <x:v>AnalysisCandidateLimit</x:v>
       </x:c>
       <x:c r="B15" t="n">
-        <x:v>50</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C15" t="str">
-        <x:v>最低表示回数</x:v>
-      </x:c>
-      <x:c r="D15" t="str"/>
+        <x:v>改善候補は最大10件</x:v>
+      </x:c>
+      <x:c r="D15"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>MinClicks</x:v>
-      </x:c>
-      <x:c r="B16" t="n">
-        <x:v>1</x:v>
+        <x:v>TodayDisplayMode</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>STEP</x:v>
       </x:c>
       <x:c r="C16" t="str">
-        <x:v>最低クリック数</x:v>
-      </x:c>
-      <x:c r="D16" t="str"/>
+        <x:v>初期2件、2件ずつ最大6件</x:v>
+      </x:c>
+      <x:c r="D16"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
-        <x:v>SearchDays</x:v>
+        <x:v>RelatedQueries</x:v>
       </x:c>
       <x:c r="B17" t="n">
-        <x:v>28</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C17" t="str">
-        <x:v>Search Console取得日数</x:v>
-      </x:c>
-      <x:c r="D17" t="str"/>
+        <x:v>改善ブリーフ用クエリ件数</x:v>
+      </x:c>
+      <x:c r="D17"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
-        <x:v>OncePerDay</x:v>
-      </x:c>
-      <x:c r="B18" t="str">
-        <x:v>ON</x:v>
+        <x:v>MinImpressions</x:v>
+      </x:c>
+      <x:c r="B18" t="n">
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C18" t="str">
-        <x:v>1日1回取得制限</x:v>
-      </x:c>
-      <x:c r="D18" t="str"/>
+        <x:v>最低表示回数</x:v>
+      </x:c>
+      <x:c r="D18"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
+        <x:v>MinClicks</x:v>
+      </x:c>
+      <x:c r="B19" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>最低クリック数</x:v>
+      </x:c>
+      <x:c r="D19"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>SearchDays</x:v>
+      </x:c>
+      <x:c r="B20" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>Search Console取得日数</x:v>
+      </x:c>
+      <x:c r="D20"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>OncePerDay</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>ON</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>1日1回取得制限</x:v>
+      </x:c>
+      <x:c r="D21"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
         <x:v>LastFetchDate</x:v>
       </x:c>
-      <x:c r="B19" t="str"/>
-      <x:c r="C19" t="str">
+      <x:c r="B22"/>
+      <x:c r="C22" t="str">
         <x:v>最終取得日</x:v>
       </x:c>
-      <x:c r="D19" t="str"/>
+      <x:c r="D22"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Improve Home dashboard and daily URL checks
</commit_message>
<xml_diff>
--- a/distribution/SIMS-Blog-Manager-template-Product5.0-Official.xlsx
+++ b/distribution/SIMS-Blog-Manager-template-Product5.0-Official.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R8816b06011ce4700"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R78f8822310f64223"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="Rdae8a45d47aa41ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R7e323f17811547c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="効果測定" sheetId="5" r:id="Re3dd538dc9c14521"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Rc301332d438d4951"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="Rf1554d820878463a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R490f0cb56ae04a74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R3592beb284ec42c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="Rcc2568e64c4c4bd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="Rb96b150dec8f4b9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R74fc838a7db74dfd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="Rb7aa3365548a4770"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="Rdb2d2ee4baa541c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="Recdb9fd8135b476e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="効果測定" sheetId="5" r:id="R2093cc50dccf4282"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Rb2890903969e4855"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="Rc475573214374c8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R1911ba42a3b242e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="Ra56f13b683b44edc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R089bf700fb124775"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R8e02a9c773c341b3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23,7 +23,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="4">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -46,8 +46,24 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFD9EAD3"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -104,6 +120,31 @@
         <x:fgColor rgb="FF5F6368"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B8043"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE6F4EA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF1F3F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDBEAFE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -112,7 +153,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="82">
+  <x:cellXfs count="101">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -297,6 +338,63 @@
     <x:xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -453,205 +551,349 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="78" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="64" t="str">
-        <x:v>SIMS-Blog-Manager</x:v>
-      </x:c>
-      <x:c r="B1" s="64" t="str">
-        <x:v>ブログ改善で迷わない。今日やることが30秒で決まる。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="33" t="str">
-        <x:v>バージョン</x:v>
-      </x:c>
-      <x:c r="B2" s="33" t="str">
-        <x:v>5.0.0-official</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="33" t="str">
-        <x:v>初回認証について</x:v>
-      </x:c>
-      <x:c r="B3" s="33" t="str">
-        <x:v>最初にApps Scriptを実行するとGoogleの承認画面が表示されます。正常な動作です。許可後、同じSTEPをもう一度実行してください。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="33" t="str"/>
-      <x:c r="B4" s="33" t="str"/>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="14" t="str">
-        <x:v>現在の状態</x:v>
-      </x:c>
-      <x:c r="B5" s="14" t="str"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="14" t="str">
-        <x:v>次にやること</x:v>
-      </x:c>
-      <x:c r="B6" s="14" t="str"/>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="33" t="str"/>
-      <x:c r="B7" s="33" t="str"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="20" t="str">
-        <x:v>今日のおすすめ改善</x:v>
-      </x:c>
-      <x:c r="B8" s="20" t="str">
-        <x:v>未作成</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="20" t="str">
-        <x:v>推定時間</x:v>
-      </x:c>
-      <x:c r="B9" s="20" t="str">
-        <x:v>-</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="20" t="str">
-        <x:v>改善候補数</x:v>
-      </x:c>
-      <x:c r="B10" s="20" t="str">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="20" t="str">
-        <x:v>本日の改善時間</x:v>
-      </x:c>
-      <x:c r="B11" s="20" t="str">
-        <x:v>30分</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="20" t="str">
-        <x:v>管理対象割合</x:v>
-      </x:c>
-      <x:c r="B12" s="20" t="str">
-        <x:v>30%</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="33" t="str"/>
-      <x:c r="B13" s="33" t="str"/>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="26" t="str">
-        <x:v>セットアップ状況</x:v>
-      </x:c>
-      <x:c r="B14" s="26" t="str">
-        <x:v>状態</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="26" t="str">
-        <x:v>STEP1 ブログ情報</x:v>
-      </x:c>
-      <x:c r="B15" s="26" t="str"/>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="26" t="str">
-        <x:v>STEP2 Google Cloud APIガイド</x:v>
-      </x:c>
-      <x:c r="B16" s="26" t="str"/>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="26" t="str">
-        <x:v>STEP3 Search Console接続</x:v>
-      </x:c>
-      <x:c r="B17" s="26" t="str"/>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="26" t="str">
-        <x:v>STEP4 初回データ取得</x:v>
-      </x:c>
-      <x:c r="B18" s="26" t="str"/>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="33" t="str"/>
-      <x:c r="B19" s="33" t="str"/>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="33" t="str">
-        <x:v>登録ブログ名</x:v>
-      </x:c>
-      <x:c r="B20" s="33" t="str"/>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="33" t="str">
+    <x:row r="1" ht="18" customHeight="1">
+      <x:c r="A1" s="91" t="str">
+        <x:v>SIMS-Blog-Manager  Home</x:v>
+      </x:c>
+      <x:c r="B1" s="91"/>
+      <x:c r="C1" s="91"/>
+      <x:c r="D1" s="91"/>
+      <x:c r="E1" s="91"/>
+      <x:c r="F1" s="91"/>
+      <x:c r="G1" s="91"/>
+      <x:c r="H1" s="92" t="str">
+        <x:v>v5.3.0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="18" customHeight="1">
+      <x:c r="A2" s="36" t="str">
+        <x:v>ブログ名</x:v>
+      </x:c>
+      <x:c r="B2" s="36" t="str">
+        <x:v>未設定</x:v>
+      </x:c>
+      <x:c r="C2" s="36"/>
+      <x:c r="D2" s="36"/>
+      <x:c r="E2" s="36" t="str">
+        <x:v>最終更新</x:v>
+      </x:c>
+      <x:c r="F2" s="36" t="str">
+        <x:v>ー</x:v>
+      </x:c>
+      <x:c r="G2" s="36"/>
+      <x:c r="H2" s="36"/>
+    </x:row>
+    <x:row r="3" ht="18" customHeight="1">
+      <x:c r="A3" s="36" t="str">
+        <x:v>総記事数</x:v>
+      </x:c>
+      <x:c r="B3" s="36" t="str">
+        <x:v>0件</x:v>
+      </x:c>
+      <x:c r="C3" s="36" t="str">
         <x:v>ブログURL</x:v>
       </x:c>
-      <x:c r="B21" s="33" t="str"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="33" t="str">
-        <x:v>Search Consoleプロパティ</x:v>
-      </x:c>
-      <x:c r="B22" s="33" t="str"/>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="33" t="str">
-        <x:v>接続状態</x:v>
-      </x:c>
-      <x:c r="B23" s="33" t="str"/>
+      <x:c r="D3" s="36"/>
+      <x:c r="E3" s="36"/>
+      <x:c r="F3" s="36"/>
+      <x:c r="G3" s="36"/>
+      <x:c r="H3" s="36"/>
+    </x:row>
+    <x:row r="4" ht="18" customHeight="1">
+      <x:c r="A4" s="36"/>
+      <x:c r="B4" s="36"/>
+      <x:c r="C4" s="36"/>
+      <x:c r="D4" s="36"/>
+      <x:c r="E4" s="36"/>
+      <x:c r="F4" s="36"/>
+      <x:c r="G4" s="36"/>
+      <x:c r="H4" s="36"/>
+    </x:row>
+    <x:row r="5" ht="18" customHeight="1">
+      <x:c r="A5" s="94" t="str">
+        <x:v>記事ランクのまとめ</x:v>
+      </x:c>
+      <x:c r="B5" s="94"/>
+      <x:c r="C5" s="94"/>
+      <x:c r="D5" s="94"/>
+      <x:c r="E5" s="94"/>
+      <x:c r="F5" s="94"/>
+      <x:c r="G5" s="94"/>
+      <x:c r="H5" s="94"/>
+    </x:row>
+    <x:row r="6" ht="18" customHeight="1">
+      <x:c r="A6" s="86" t="str">
+        <x:v>🏆 エース</x:v>
+      </x:c>
+      <x:c r="B6" s="86"/>
+      <x:c r="C6" s="36" t="str">
+        <x:v>✅ 安定</x:v>
+      </x:c>
+      <x:c r="D6" s="36"/>
+      <x:c r="E6" s="36" t="str">
+        <x:v>📈 成長</x:v>
+      </x:c>
+      <x:c r="F6" s="36"/>
+      <x:c r="G6" s="36" t="str">
+        <x:v>🌱 育成</x:v>
+      </x:c>
+      <x:c r="H6" s="36"/>
+    </x:row>
+    <x:row r="7" ht="18" customHeight="1">
+      <x:c r="A7" s="36" t="str">
+        <x:v>0件 →</x:v>
+      </x:c>
+      <x:c r="B7" s="36"/>
+      <x:c r="C7" s="36" t="str">
+        <x:v>0件 →</x:v>
+      </x:c>
+      <x:c r="D7" s="36"/>
+      <x:c r="E7" s="36" t="str">
+        <x:v>0件 →</x:v>
+      </x:c>
+      <x:c r="F7" s="36"/>
+      <x:c r="G7" s="36" t="str">
+        <x:v>0件 →</x:v>
+      </x:c>
+      <x:c r="H7" s="36"/>
+    </x:row>
+    <x:row r="8" ht="18" customHeight="1">
+      <x:c r="A8" s="87" t="str">
+        <x:v>⚠️ 低迷</x:v>
+      </x:c>
+      <x:c r="B8" s="87"/>
+      <x:c r="C8" s="36" t="str">
+        <x:v>ブログの現在地</x:v>
+      </x:c>
+      <x:c r="D8" s="36"/>
+      <x:c r="E8" s="36"/>
+      <x:c r="F8" s="36"/>
+      <x:c r="G8" s="36"/>
+      <x:c r="H8" s="36"/>
+    </x:row>
+    <x:row r="9" ht="18" customHeight="1">
+      <x:c r="A9" s="87" t="str">
+        <x:v>0件 →</x:v>
+      </x:c>
+      <x:c r="B9" s="87"/>
+      <x:c r="C9" s="36" t="str">
+        <x:v>記事データを分析しています。</x:v>
+      </x:c>
+      <x:c r="D9" s="36"/>
+      <x:c r="E9" s="36"/>
+      <x:c r="F9" s="36"/>
+      <x:c r="G9" s="36"/>
+      <x:c r="H9" s="36"/>
+    </x:row>
+    <x:row r="10" ht="18" customHeight="1">
+      <x:c r="A10" s="87"/>
+      <x:c r="B10" s="87"/>
+      <x:c r="C10" s="36"/>
+      <x:c r="D10" s="36"/>
+      <x:c r="E10" s="36"/>
+      <x:c r="F10" s="36"/>
+      <x:c r="G10" s="36"/>
+      <x:c r="H10" s="36"/>
+    </x:row>
+    <x:row r="11" ht="18" customHeight="1">
+      <x:c r="A11" s="96" t="str">
+        <x:v>改善状況</x:v>
+      </x:c>
+      <x:c r="B11" s="96"/>
+      <x:c r="C11" s="96"/>
+      <x:c r="D11" s="96"/>
+      <x:c r="E11" s="96"/>
+      <x:c r="F11" s="96"/>
+      <x:c r="G11" s="96"/>
+      <x:c r="H11" s="96"/>
+    </x:row>
+    <x:row r="12" ht="18" customHeight="1">
+      <x:c r="A12" s="87" t="str">
+        <x:v>今日の改善</x:v>
+      </x:c>
+      <x:c r="B12" s="87"/>
+      <x:c r="C12" s="36" t="str">
+        <x:v>改善中</x:v>
+      </x:c>
+      <x:c r="D12" s="36"/>
+      <x:c r="E12" s="36" t="str">
+        <x:v>効果測定中</x:v>
+      </x:c>
+      <x:c r="F12" s="36"/>
+      <x:c r="G12" s="36" t="str">
+        <x:v>要確認</x:v>
+      </x:c>
+      <x:c r="H12" s="36"/>
+    </x:row>
+    <x:row r="13" ht="18" customHeight="1">
+      <x:c r="A13" s="36" t="str">
+        <x:v>0件</x:v>
+      </x:c>
+      <x:c r="B13" s="36"/>
+      <x:c r="C13" s="36" t="str">
+        <x:v>0件</x:v>
+      </x:c>
+      <x:c r="D13" s="36"/>
+      <x:c r="E13" s="36" t="str">
+        <x:v>0件</x:v>
+      </x:c>
+      <x:c r="F13" s="36"/>
+      <x:c r="G13" s="36" t="str">
+        <x:v>0件</x:v>
+      </x:c>
+      <x:c r="H13" s="36"/>
+    </x:row>
+    <x:row r="14" ht="18" customHeight="1">
+      <x:c r="A14" s="88"/>
+      <x:c r="B14" s="88"/>
+      <x:c r="C14" s="36"/>
+      <x:c r="D14" s="36"/>
+      <x:c r="E14" s="36"/>
+      <x:c r="F14" s="36"/>
+      <x:c r="G14" s="36"/>
+      <x:c r="H14" s="36"/>
+    </x:row>
+    <x:row r="15" ht="18" customHeight="1">
+      <x:c r="A15" s="98" t="str">
+        <x:v>今日のメッセージ</x:v>
+      </x:c>
+      <x:c r="B15" s="98"/>
+      <x:c r="C15" s="98"/>
+      <x:c r="D15" s="98"/>
+      <x:c r="E15" s="98"/>
+      <x:c r="F15" s="98"/>
+      <x:c r="G15" s="98"/>
+      <x:c r="H15" s="98"/>
+    </x:row>
+    <x:row r="16" ht="18" customHeight="1">
+      <x:c r="A16" s="88" t="str">
+        <x:v>記事の育ち方と改善状況に合わせて表示します。</x:v>
+      </x:c>
+      <x:c r="B16" s="88"/>
+      <x:c r="C16" s="36"/>
+      <x:c r="D16" s="36"/>
+      <x:c r="E16" s="36"/>
+      <x:c r="F16" s="36"/>
+      <x:c r="G16" s="36"/>
+      <x:c r="H16" s="36"/>
+    </x:row>
+    <x:row r="17" ht="18" customHeight="1">
+      <x:c r="A17" s="88"/>
+      <x:c r="B17" s="88"/>
+      <x:c r="C17" s="36"/>
+      <x:c r="D17" s="36"/>
+      <x:c r="E17" s="36"/>
+      <x:c r="F17" s="36"/>
+      <x:c r="G17" s="36"/>
+      <x:c r="H17" s="36"/>
+    </x:row>
+    <x:row r="18" ht="18" customHeight="1">
+      <x:c r="A18" s="88"/>
+      <x:c r="B18" s="88"/>
+      <x:c r="C18" s="36"/>
+      <x:c r="D18" s="36"/>
+      <x:c r="E18" s="36"/>
+      <x:c r="F18" s="36"/>
+      <x:c r="G18" s="36"/>
+      <x:c r="H18" s="36"/>
+    </x:row>
+    <x:row r="19" ht="18" customHeight="1">
+      <x:c r="A19" s="36" t="str">
+        <x:v>処理状況</x:v>
+      </x:c>
+      <x:c r="B19" s="36"/>
+      <x:c r="C19" s="36"/>
+      <x:c r="D19" s="36"/>
+      <x:c r="E19" s="36"/>
+      <x:c r="F19" s="36"/>
+      <x:c r="G19" s="36"/>
+      <x:c r="H19" s="36"/>
+    </x:row>
+    <x:row r="20" ht="18" customHeight="1">
+      <x:c r="A20" s="100" t="str">
+        <x:v>処理名</x:v>
+      </x:c>
+      <x:c r="B20" s="100"/>
+      <x:c r="C20" s="100"/>
+      <x:c r="D20" s="100"/>
+      <x:c r="E20" s="100"/>
+      <x:c r="F20" s="100"/>
+      <x:c r="G20" s="100"/>
+      <x:c r="H20" s="100"/>
+    </x:row>
+    <x:row r="21" ht="18" customHeight="1">
+      <x:c r="A21" s="99" t="str">
+        <x:v>開始時刻</x:v>
+      </x:c>
+      <x:c r="B21" s="99"/>
+      <x:c r="C21" s="99"/>
+      <x:c r="D21" s="99" t="str">
+        <x:v>処理結果</x:v>
+      </x:c>
+      <x:c r="E21" s="99"/>
+      <x:c r="F21" s="99"/>
+      <x:c r="G21" s="99"/>
+      <x:c r="H21" s="99"/>
+    </x:row>
+    <x:row r="22" ht="18" customHeight="1">
+      <x:c r="A22" s="99" t="str">
+        <x:v>お願い</x:v>
+      </x:c>
+      <x:c r="B22" s="99"/>
+      <x:c r="C22" s="99"/>
+      <x:c r="D22" s="99"/>
+      <x:c r="E22" s="99"/>
+      <x:c r="F22" s="99"/>
+      <x:c r="G22" s="99"/>
+      <x:c r="H22" s="99"/>
+    </x:row>
+    <x:row r="23" ht="18" customHeight="1">
+      <x:c r="A23" s="99"/>
+      <x:c r="B23" s="99"/>
+      <x:c r="C23" s="99"/>
+      <x:c r="D23" s="99"/>
+      <x:c r="E23" s="99"/>
+      <x:c r="F23" s="99"/>
+      <x:c r="G23" s="99"/>
+      <x:c r="H23" s="99"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="33" t="str">
-        <x:v>最終取得日</x:v>
-      </x:c>
-      <x:c r="B24" s="33" t="str"/>
+      <x:c r="A24" s="33"/>
+      <x:c r="B24" s="33"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="33" t="str"/>
-      <x:c r="B25" s="33" t="str"/>
+      <x:c r="A25" s="33"/>
+      <x:c r="B25" s="33"/>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="33" t="str">
-        <x:v>最近の成果</x:v>
-      </x:c>
-      <x:c r="B26" s="33" t="str"/>
+      <x:c r="A26" s="33"/>
+      <x:c r="B26" s="33"/>
     </x:row>
     <x:row r="27">
-      <x:c r="A27" s="28" t="str">
-        <x:v>成功</x:v>
-      </x:c>
-      <x:c r="B27" s="28" t="str">
-        <x:v>0件</x:v>
-      </x:c>
+      <x:c r="A27" s="28"/>
+      <x:c r="B27" s="28"/>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="28" t="str">
-        <x:v>横ばい</x:v>
-      </x:c>
-      <x:c r="B28" s="28" t="str">
-        <x:v>0件</x:v>
-      </x:c>
+      <x:c r="A28" s="28"/>
+      <x:c r="B28" s="28"/>
     </x:row>
     <x:row r="29">
-      <x:c r="A29" s="28" t="str">
-        <x:v>要再改善</x:v>
-      </x:c>
-      <x:c r="B29" s="28" t="str">
-        <x:v>0件</x:v>
-      </x:c>
+      <x:c r="A29" s="28"/>
+      <x:c r="B29" s="28"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="28" t="str">
-        <x:v>測定待ち</x:v>
-      </x:c>
-      <x:c r="B30" s="28" t="str">
-        <x:v>0件</x:v>
-      </x:c>
+      <x:c r="A30" s="28"/>
+      <x:c r="B30" s="28"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="28" t="str"/>
@@ -666,6 +908,41 @@
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="B2:D2"/>
+    <x:mergeCell ref="F2:H2"/>
+    <x:mergeCell ref="D3:H3"/>
+    <x:mergeCell ref="A5:H5"/>
+    <x:mergeCell ref="A6:B6"/>
+    <x:mergeCell ref="C6:D6"/>
+    <x:mergeCell ref="E6:F6"/>
+    <x:mergeCell ref="G6:H6"/>
+    <x:mergeCell ref="A7:B7"/>
+    <x:mergeCell ref="C7:D7"/>
+    <x:mergeCell ref="E7:F7"/>
+    <x:mergeCell ref="G7:H7"/>
+    <x:mergeCell ref="A8:B8"/>
+    <x:mergeCell ref="C8:H8"/>
+    <x:mergeCell ref="A9:B9"/>
+    <x:mergeCell ref="C9:H9"/>
+    <x:mergeCell ref="A11:H11"/>
+    <x:mergeCell ref="A12:B12"/>
+    <x:mergeCell ref="C12:D12"/>
+    <x:mergeCell ref="E12:F12"/>
+    <x:mergeCell ref="G12:H12"/>
+    <x:mergeCell ref="A13:B13"/>
+    <x:mergeCell ref="C13:D13"/>
+    <x:mergeCell ref="E13:F13"/>
+    <x:mergeCell ref="G13:H13"/>
+    <x:mergeCell ref="A15:H15"/>
+    <x:mergeCell ref="A16:H18"/>
+    <x:mergeCell ref="A20:H20"/>
+    <x:mergeCell ref="B21:H21"/>
+    <x:mergeCell ref="B22:C22"/>
+    <x:mergeCell ref="E22:H22"/>
+    <x:mergeCell ref="B23:H23"/>
+  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Redesign menus around user actions
</commit_message>
<xml_diff>
--- a/distribution/SIMS-Blog-Manager-template-Product5.0-Official.xlsx
+++ b/distribution/SIMS-Blog-Manager-template-Product5.0-Official.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R74fc838a7db74dfd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="Rb7aa3365548a4770"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="Rdb2d2ee4baa541c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="Recdb9fd8135b476e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="効果測定" sheetId="5" r:id="R2093cc50dccf4282"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="Rb2890903969e4855"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="Rc475573214374c8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R1911ba42a3b242e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="Ra56f13b683b44edc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R089bf700fb124775"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="R8e02a9c773c341b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="Rd0f743e0c6e840e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R1928a7e33b2f4f8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="R07b9b7bedd8f43b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R46ac6f6db47c4288"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="効果測定" sheetId="5" r:id="Rf66c5c855ace46d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="R19d76b30bca34311"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="Rb5483bff278147fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="Rab0b3a63bbf647a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R1bdfb9b33e0a4851"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R4b176dc287e5424a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="Ra6a1ce5f913f4713"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -63,7 +63,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="17">
+  <x:fills count="22">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -145,6 +145,31 @@
         <x:fgColor rgb="FFD9EAD3"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B8043"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE6F4EA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF1F3F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDBEAFE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -153,7 +178,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="101">
+  <x:cellXfs count="123">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -395,6 +420,72 @@
     <x:xf numFmtId="0" fontId="6" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -562,17 +653,17 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="18" customHeight="1">
-      <x:c r="A1" s="91" t="str">
+      <x:c r="A1" s="105" t="str">
         <x:v>SIMS-Blog-Manager  Home</x:v>
       </x:c>
-      <x:c r="B1" s="91"/>
-      <x:c r="C1" s="91"/>
-      <x:c r="D1" s="91"/>
-      <x:c r="E1" s="91"/>
-      <x:c r="F1" s="91"/>
-      <x:c r="G1" s="91"/>
-      <x:c r="H1" s="92" t="str">
-        <x:v>v5.3.0</x:v>
+      <x:c r="B1" s="105"/>
+      <x:c r="C1" s="105"/>
+      <x:c r="D1" s="105"/>
+      <x:c r="E1" s="105"/>
+      <x:c r="F1" s="105"/>
+      <x:c r="G1" s="105"/>
+      <x:c r="H1" s="106" t="str">
+        <x:v>v5.3.1</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="18" customHeight="1">
@@ -620,175 +711,173 @@
       <x:c r="H4" s="36"/>
     </x:row>
     <x:row r="5" ht="18" customHeight="1">
-      <x:c r="A5" s="94" t="str">
+      <x:c r="A5" s="107" t="str">
         <x:v>記事ランクのまとめ</x:v>
       </x:c>
-      <x:c r="B5" s="94"/>
-      <x:c r="C5" s="94"/>
-      <x:c r="D5" s="94"/>
-      <x:c r="E5" s="94"/>
-      <x:c r="F5" s="94"/>
-      <x:c r="G5" s="94"/>
-      <x:c r="H5" s="94"/>
+      <x:c r="B5" s="107"/>
+      <x:c r="C5" s="107"/>
+      <x:c r="D5" s="107"/>
+      <x:c r="E5" s="107"/>
+      <x:c r="F5" s="107"/>
+      <x:c r="G5" s="107"/>
+      <x:c r="H5" s="107"/>
     </x:row>
     <x:row r="6" ht="18" customHeight="1">
-      <x:c r="A6" s="86" t="str">
+      <x:c r="A6" s="114" t="str">
         <x:v>🏆 エース</x:v>
       </x:c>
-      <x:c r="B6" s="86"/>
-      <x:c r="C6" s="36" t="str">
+      <x:c r="B6" s="114"/>
+      <x:c r="C6" s="115"/>
+      <x:c r="D6" s="115"/>
+      <x:c r="E6" s="115" t="str">
         <x:v>✅ 安定</x:v>
       </x:c>
-      <x:c r="D6" s="36"/>
-      <x:c r="E6" s="36" t="str">
+      <x:c r="F6" s="115"/>
+      <x:c r="G6" s="115"/>
+      <x:c r="H6" s="115"/>
+    </x:row>
+    <x:row r="7" ht="18" customHeight="1">
+      <x:c r="A7" s="115" t="str">
+        <x:v>0件 →</x:v>
+      </x:c>
+      <x:c r="B7" s="115"/>
+      <x:c r="C7" s="115"/>
+      <x:c r="D7" s="115"/>
+      <x:c r="E7" s="115" t="str">
+        <x:v>0件 →</x:v>
+      </x:c>
+      <x:c r="F7" s="115"/>
+      <x:c r="G7" s="115"/>
+      <x:c r="H7" s="115"/>
+    </x:row>
+    <x:row r="8" ht="18" customHeight="1">
+      <x:c r="A8" s="116" t="str">
         <x:v>📈 成長</x:v>
       </x:c>
-      <x:c r="F6" s="36"/>
-      <x:c r="G6" s="36" t="str">
+      <x:c r="B8" s="116"/>
+      <x:c r="C8" s="115"/>
+      <x:c r="D8" s="115"/>
+      <x:c r="E8" s="115" t="str">
         <x:v>🌱 育成</x:v>
       </x:c>
-      <x:c r="H6" s="36"/>
-    </x:row>
-    <x:row r="7" ht="18" customHeight="1">
-      <x:c r="A7" s="36" t="str">
+      <x:c r="F8" s="115"/>
+      <x:c r="G8" s="115"/>
+      <x:c r="H8" s="115"/>
+    </x:row>
+    <x:row r="9" ht="18" customHeight="1">
+      <x:c r="A9" s="116" t="str">
         <x:v>0件 →</x:v>
       </x:c>
-      <x:c r="B7" s="36"/>
-      <x:c r="C7" s="36" t="str">
+      <x:c r="B9" s="116"/>
+      <x:c r="C9" s="115"/>
+      <x:c r="D9" s="115"/>
+      <x:c r="E9" s="115" t="str">
         <x:v>0件 →</x:v>
       </x:c>
-      <x:c r="D7" s="36"/>
-      <x:c r="E7" s="36" t="str">
-        <x:v>0件 →</x:v>
-      </x:c>
-      <x:c r="F7" s="36"/>
-      <x:c r="G7" s="36" t="str">
-        <x:v>0件 →</x:v>
-      </x:c>
-      <x:c r="H7" s="36"/>
-    </x:row>
-    <x:row r="8" ht="18" customHeight="1">
-      <x:c r="A8" s="87" t="str">
+      <x:c r="F9" s="115"/>
+      <x:c r="G9" s="115"/>
+      <x:c r="H9" s="115"/>
+    </x:row>
+    <x:row r="10" ht="18" customHeight="1">
+      <x:c r="A10" s="116" t="str">
         <x:v>⚠️ 低迷</x:v>
       </x:c>
-      <x:c r="B8" s="87"/>
-      <x:c r="C8" s="36" t="str">
-        <x:v>ブログの現在地</x:v>
-      </x:c>
-      <x:c r="D8" s="36"/>
-      <x:c r="E8" s="36"/>
-      <x:c r="F8" s="36"/>
-      <x:c r="G8" s="36"/>
-      <x:c r="H8" s="36"/>
-    </x:row>
-    <x:row r="9" ht="18" customHeight="1">
-      <x:c r="A9" s="87" t="str">
-        <x:v>0件 →</x:v>
-      </x:c>
-      <x:c r="B9" s="87"/>
-      <x:c r="C9" s="36" t="str">
-        <x:v>記事データを分析しています。</x:v>
-      </x:c>
-      <x:c r="D9" s="36"/>
-      <x:c r="E9" s="36"/>
-      <x:c r="F9" s="36"/>
-      <x:c r="G9" s="36"/>
-      <x:c r="H9" s="36"/>
-    </x:row>
-    <x:row r="10" ht="18" customHeight="1">
-      <x:c r="A10" s="87"/>
-      <x:c r="B10" s="87"/>
-      <x:c r="C10" s="36"/>
-      <x:c r="D10" s="36"/>
-      <x:c r="E10" s="36"/>
-      <x:c r="F10" s="36"/>
-      <x:c r="G10" s="36"/>
-      <x:c r="H10" s="36"/>
+      <x:c r="B10" s="116"/>
+      <x:c r="C10" s="115"/>
+      <x:c r="D10" s="115"/>
+      <x:c r="E10" s="115" t="str">
+        <x:v>❓ 未取得</x:v>
+      </x:c>
+      <x:c r="F10" s="115"/>
+      <x:c r="G10" s="115"/>
+      <x:c r="H10" s="115"/>
     </x:row>
     <x:row r="11" ht="18" customHeight="1">
       <x:c r="A11" s="96" t="str">
-        <x:v>改善状況</x:v>
+        <x:v>0件 →</x:v>
       </x:c>
       <x:c r="B11" s="96"/>
       <x:c r="C11" s="96"/>
       <x:c r="D11" s="96"/>
-      <x:c r="E11" s="96"/>
+      <x:c r="E11" s="96" t="str">
+        <x:v>0件 →</x:v>
+      </x:c>
       <x:c r="F11" s="96"/>
       <x:c r="G11" s="96"/>
       <x:c r="H11" s="96"/>
     </x:row>
     <x:row r="12" ht="18" customHeight="1">
-      <x:c r="A12" s="87" t="str">
-        <x:v>今日の改善</x:v>
-      </x:c>
-      <x:c r="B12" s="87"/>
-      <x:c r="C12" s="36" t="str">
-        <x:v>改善中</x:v>
-      </x:c>
-      <x:c r="D12" s="36"/>
-      <x:c r="E12" s="36" t="str">
-        <x:v>効果測定中</x:v>
-      </x:c>
-      <x:c r="F12" s="36"/>
-      <x:c r="G12" s="36" t="str">
-        <x:v>要確認</x:v>
-      </x:c>
-      <x:c r="H12" s="36"/>
+      <x:c r="A12" s="118"/>
+      <x:c r="B12" s="118"/>
+      <x:c r="C12" s="118"/>
+      <x:c r="D12" s="118"/>
+      <x:c r="E12" s="118"/>
+      <x:c r="F12" s="118"/>
+      <x:c r="G12" s="118"/>
+      <x:c r="H12" s="118"/>
     </x:row>
     <x:row r="13" ht="18" customHeight="1">
       <x:c r="A13" s="36" t="str">
-        <x:v>0件</x:v>
+        <x:v>改善状況</x:v>
       </x:c>
       <x:c r="B13" s="36"/>
-      <x:c r="C13" s="36" t="str">
-        <x:v>0件</x:v>
-      </x:c>
+      <x:c r="C13" s="36"/>
       <x:c r="D13" s="36"/>
-      <x:c r="E13" s="36" t="str">
-        <x:v>0件</x:v>
-      </x:c>
+      <x:c r="E13" s="36"/>
       <x:c r="F13" s="36"/>
-      <x:c r="G13" s="36" t="str">
-        <x:v>0件</x:v>
-      </x:c>
+      <x:c r="G13" s="36"/>
       <x:c r="H13" s="36"/>
     </x:row>
     <x:row r="14" ht="18" customHeight="1">
-      <x:c r="A14" s="88"/>
+      <x:c r="A14" s="88" t="str">
+        <x:v>今日の改善</x:v>
+      </x:c>
       <x:c r="B14" s="88"/>
-      <x:c r="C14" s="36"/>
+      <x:c r="C14" s="36" t="str">
+        <x:v>改善中</x:v>
+      </x:c>
       <x:c r="D14" s="36"/>
-      <x:c r="E14" s="36"/>
+      <x:c r="E14" s="36" t="str">
+        <x:v>効果測定中</x:v>
+      </x:c>
       <x:c r="F14" s="36"/>
-      <x:c r="G14" s="36"/>
+      <x:c r="G14" s="36" t="str">
+        <x:v>要確認</x:v>
+      </x:c>
       <x:c r="H14" s="36"/>
     </x:row>
     <x:row r="15" ht="18" customHeight="1">
       <x:c r="A15" s="98" t="str">
+        <x:v>0件</x:v>
+      </x:c>
+      <x:c r="B15" s="98"/>
+      <x:c r="C15" s="98" t="str">
+        <x:v>0件</x:v>
+      </x:c>
+      <x:c r="D15" s="98"/>
+      <x:c r="E15" s="98" t="str">
+        <x:v>0件</x:v>
+      </x:c>
+      <x:c r="F15" s="98"/>
+      <x:c r="G15" s="98" t="str">
+        <x:v>0件</x:v>
+      </x:c>
+      <x:c r="H15" s="98"/>
+    </x:row>
+    <x:row r="16" ht="18" customHeight="1">
+      <x:c r="A16" s="120"/>
+      <x:c r="B16" s="120"/>
+      <x:c r="C16" s="120"/>
+      <x:c r="D16" s="120"/>
+      <x:c r="E16" s="120"/>
+      <x:c r="F16" s="120"/>
+      <x:c r="G16" s="120"/>
+      <x:c r="H16" s="120"/>
+    </x:row>
+    <x:row r="17" ht="18" customHeight="1">
+      <x:c r="A17" s="88" t="str">
         <x:v>今日のメッセージ</x:v>
       </x:c>
-      <x:c r="B15" s="98"/>
-      <x:c r="C15" s="98"/>
-      <x:c r="D15" s="98"/>
-      <x:c r="E15" s="98"/>
-      <x:c r="F15" s="98"/>
-      <x:c r="G15" s="98"/>
-      <x:c r="H15" s="98"/>
-    </x:row>
-    <x:row r="16" ht="18" customHeight="1">
-      <x:c r="A16" s="88" t="str">
-        <x:v>記事の育ち方と改善状況に合わせて表示します。</x:v>
-      </x:c>
-      <x:c r="B16" s="88"/>
-      <x:c r="C16" s="36"/>
-      <x:c r="D16" s="36"/>
-      <x:c r="E16" s="36"/>
-      <x:c r="F16" s="36"/>
-      <x:c r="G16" s="36"/>
-      <x:c r="H16" s="36"/>
-    </x:row>
-    <x:row r="17" ht="18" customHeight="1">
-      <x:c r="A17" s="88"/>
       <x:c r="B17" s="88"/>
       <x:c r="C17" s="36"/>
       <x:c r="D17" s="36"/>
@@ -798,7 +887,9 @@
       <x:c r="H17" s="36"/>
     </x:row>
     <x:row r="18" ht="18" customHeight="1">
-      <x:c r="A18" s="88"/>
+      <x:c r="A18" s="88" t="str">
+        <x:v>記事の育ち方と改善状況に合わせて表示します。</x:v>
+      </x:c>
       <x:c r="B18" s="88"/>
       <x:c r="C18" s="36"/>
       <x:c r="D18" s="36"/>
@@ -808,9 +899,7 @@
       <x:c r="H18" s="36"/>
     </x:row>
     <x:row r="19" ht="18" customHeight="1">
-      <x:c r="A19" s="36" t="str">
-        <x:v>処理状況</x:v>
-      </x:c>
+      <x:c r="A19" s="36"/>
       <x:c r="B19" s="36"/>
       <x:c r="C19" s="36"/>
       <x:c r="D19" s="36"/>
@@ -820,9 +909,7 @@
       <x:c r="H19" s="36"/>
     </x:row>
     <x:row r="20" ht="18" customHeight="1">
-      <x:c r="A20" s="100" t="str">
-        <x:v>処理名</x:v>
-      </x:c>
+      <x:c r="A20" s="100"/>
       <x:c r="B20" s="100"/>
       <x:c r="C20" s="100"/>
       <x:c r="D20" s="100"/>
@@ -832,44 +919,54 @@
       <x:c r="H20" s="100"/>
     </x:row>
     <x:row r="21" ht="18" customHeight="1">
-      <x:c r="A21" s="99" t="str">
+      <x:c r="A21" s="122" t="str">
+        <x:v>処理状況</x:v>
+      </x:c>
+      <x:c r="B21" s="122"/>
+      <x:c r="C21" s="122"/>
+      <x:c r="D21" s="122"/>
+      <x:c r="E21" s="122"/>
+      <x:c r="F21" s="122"/>
+      <x:c r="G21" s="122"/>
+      <x:c r="H21" s="122"/>
+    </x:row>
+    <x:row r="22" ht="18" customHeight="1">
+      <x:c r="A22" s="121" t="str">
+        <x:v>処理名</x:v>
+      </x:c>
+      <x:c r="B22" s="121"/>
+      <x:c r="C22" s="121"/>
+      <x:c r="D22" s="121"/>
+      <x:c r="E22" s="121"/>
+      <x:c r="F22" s="121"/>
+      <x:c r="G22" s="121"/>
+      <x:c r="H22" s="121"/>
+    </x:row>
+    <x:row r="23" ht="18" customHeight="1">
+      <x:c r="A23" s="121" t="str">
         <x:v>開始時刻</x:v>
       </x:c>
-      <x:c r="B21" s="99"/>
-      <x:c r="C21" s="99"/>
-      <x:c r="D21" s="99" t="str">
+      <x:c r="B23" s="121"/>
+      <x:c r="C23" s="121"/>
+      <x:c r="D23" s="121" t="str">
         <x:v>処理結果</x:v>
       </x:c>
-      <x:c r="E21" s="99"/>
-      <x:c r="F21" s="99"/>
-      <x:c r="G21" s="99"/>
-      <x:c r="H21" s="99"/>
-    </x:row>
-    <x:row r="22" ht="18" customHeight="1">
-      <x:c r="A22" s="99" t="str">
+      <x:c r="E23" s="121"/>
+      <x:c r="F23" s="121"/>
+      <x:c r="G23" s="121"/>
+      <x:c r="H23" s="121"/>
+    </x:row>
+    <x:row r="24" ht="18" customHeight="1">
+      <x:c r="A24" s="121" t="str">
         <x:v>お願い</x:v>
       </x:c>
-      <x:c r="B22" s="99"/>
-      <x:c r="C22" s="99"/>
-      <x:c r="D22" s="99"/>
-      <x:c r="E22" s="99"/>
-      <x:c r="F22" s="99"/>
-      <x:c r="G22" s="99"/>
-      <x:c r="H22" s="99"/>
-    </x:row>
-    <x:row r="23" ht="18" customHeight="1">
-      <x:c r="A23" s="99"/>
-      <x:c r="B23" s="99"/>
-      <x:c r="C23" s="99"/>
-      <x:c r="D23" s="99"/>
-      <x:c r="E23" s="99"/>
-      <x:c r="F23" s="99"/>
-      <x:c r="G23" s="99"/>
-      <x:c r="H23" s="99"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="33"/>
-      <x:c r="B24" s="33"/>
+      <x:c r="B24" s="121"/>
+      <x:c r="C24" s="121"/>
+      <x:c r="D24" s="121"/>
+      <x:c r="E24" s="121"/>
+      <x:c r="F24" s="121"/>
+      <x:c r="G24" s="121"/>
+      <x:c r="H24" s="121"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="33"/>
@@ -942,6 +1039,28 @@
     <x:mergeCell ref="B22:C22"/>
     <x:mergeCell ref="E22:H22"/>
     <x:mergeCell ref="B23:H23"/>
+    <x:mergeCell ref="A6:D6"/>
+    <x:mergeCell ref="E6:H6"/>
+    <x:mergeCell ref="A7:D7"/>
+    <x:mergeCell ref="E7:H7"/>
+    <x:mergeCell ref="A8:D8"/>
+    <x:mergeCell ref="E8:H8"/>
+    <x:mergeCell ref="A9:D9"/>
+    <x:mergeCell ref="E9:H9"/>
+    <x:mergeCell ref="A10:D10"/>
+    <x:mergeCell ref="E10:H10"/>
+    <x:mergeCell ref="A12:H12"/>
+    <x:mergeCell ref="A14:B14"/>
+    <x:mergeCell ref="C14:D14"/>
+    <x:mergeCell ref="E14:F14"/>
+    <x:mergeCell ref="G14:H14"/>
+    <x:mergeCell ref="A16:H16"/>
+    <x:mergeCell ref="A17:H19"/>
+    <x:mergeCell ref="A21:H21"/>
+    <x:mergeCell ref="B22:H22"/>
+    <x:mergeCell ref="B23:C23"/>
+    <x:mergeCell ref="E23:H23"/>
+    <x:mergeCell ref="B24:H24"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Fix Home ranks and restore detail actions
</commit_message>
<xml_diff>
--- a/distribution/SIMS-Blog-Manager-template-Product5.0-Official.xlsx
+++ b/distribution/SIMS-Blog-Manager-template-Product5.0-Official.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="Rd0f743e0c6e840e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="R1928a7e33b2f4f8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="R07b9b7bedd8f43b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R46ac6f6db47c4288"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="効果測定" sheetId="5" r:id="Rf66c5c855ace46d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="R19d76b30bca34311"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="Rb5483bff278147fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="Rab0b3a63bbf647a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R1bdfb9b33e0a4851"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R4b176dc287e5424a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="Ra6a1ce5f913f4713"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ホーム" sheetId="1" r:id="R92bab31fce614ab4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="今日の改善" sheetId="2" r:id="Ra9eec4d2f3d1405e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ログ" sheetId="3" r:id="R6f751e86df0046c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="セットアップ" sheetId="4" r:id="R38217a800fc14209"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善の推移" sheetId="5" r:id="R7aeacc338c1e4ee6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="改善ブリーフ" sheetId="6" r:id="R75ed926acf354778"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="7" r:id="Rc26107cb6c894389"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="System_Log" sheetId="8" r:id="R97351f6036514090"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="クエリデータ" sheetId="9" r:id="R4f0fd09d520e46e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事カルテ" sheetId="10" r:id="R90dd264dbe684fb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="記事診断" sheetId="11" r:id="Ra74a72e283d6454f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -63,7 +63,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="22">
+  <x:fills count="29">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -170,6 +170,41 @@
         <x:fgColor rgb="FFD9EAD3"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B8043"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE6F4EA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F8F3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF8E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF1F3F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDBEAFE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAD3"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -178,7 +213,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="123">
+  <x:cellXfs count="134">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -486,6 +521,39 @@
     <x:xf numFmtId="0" fontId="6" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -653,17 +721,17 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="18" customHeight="1">
-      <x:c r="A1" s="105" t="str">
+      <x:c r="A1" s="123" t="str">
         <x:v>SIMS-Blog-Manager  Home</x:v>
       </x:c>
-      <x:c r="B1" s="105"/>
-      <x:c r="C1" s="105"/>
-      <x:c r="D1" s="105"/>
-      <x:c r="E1" s="105"/>
-      <x:c r="F1" s="105"/>
-      <x:c r="G1" s="105"/>
-      <x:c r="H1" s="106" t="str">
-        <x:v>v5.3.1</x:v>
+      <x:c r="B1" s="123"/>
+      <x:c r="C1" s="123"/>
+      <x:c r="D1" s="123"/>
+      <x:c r="E1" s="123"/>
+      <x:c r="F1" s="123"/>
+      <x:c r="G1" s="123"/>
+      <x:c r="H1" s="124" t="str">
+        <x:v>v5.3.2</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="18" customHeight="1">
@@ -711,122 +779,122 @@
       <x:c r="H4" s="36"/>
     </x:row>
     <x:row r="5" ht="18" customHeight="1">
-      <x:c r="A5" s="107" t="str">
+      <x:c r="A5" s="125" t="str">
         <x:v>記事ランクのまとめ</x:v>
       </x:c>
-      <x:c r="B5" s="107"/>
-      <x:c r="C5" s="107"/>
-      <x:c r="D5" s="107"/>
-      <x:c r="E5" s="107"/>
-      <x:c r="F5" s="107"/>
-      <x:c r="G5" s="107"/>
-      <x:c r="H5" s="107"/>
+      <x:c r="B5" s="125"/>
+      <x:c r="C5" s="125"/>
+      <x:c r="D5" s="125"/>
+      <x:c r="E5" s="125"/>
+      <x:c r="F5" s="125"/>
+      <x:c r="G5" s="125"/>
+      <x:c r="H5" s="125"/>
     </x:row>
     <x:row r="6" ht="18" customHeight="1">
-      <x:c r="A6" s="114" t="str">
+      <x:c r="A6" s="126" t="str">
         <x:v>🏆 エース</x:v>
       </x:c>
-      <x:c r="B6" s="114"/>
-      <x:c r="C6" s="115"/>
-      <x:c r="D6" s="115"/>
-      <x:c r="E6" s="115" t="str">
+      <x:c r="B6" s="126"/>
+      <x:c r="C6" s="126" t="str">
+        <x:v>0件 →</x:v>
+      </x:c>
+      <x:c r="D6" s="126"/>
+      <x:c r="E6" s="127" t="str">
+        <x:v>🌱 育成</x:v>
+      </x:c>
+      <x:c r="F6" s="127"/>
+      <x:c r="G6" s="127" t="str">
+        <x:v>0件 →</x:v>
+      </x:c>
+      <x:c r="H6" s="127"/>
+    </x:row>
+    <x:row r="7" ht="18" customHeight="1">
+      <x:c r="A7" s="126" t="str">
         <x:v>✅ 安定</x:v>
       </x:c>
-      <x:c r="F6" s="115"/>
-      <x:c r="G6" s="115"/>
-      <x:c r="H6" s="115"/>
-    </x:row>
-    <x:row r="7" ht="18" customHeight="1">
-      <x:c r="A7" s="115" t="str">
+      <x:c r="B7" s="126"/>
+      <x:c r="C7" s="126" t="str">
         <x:v>0件 →</x:v>
       </x:c>
-      <x:c r="B7" s="115"/>
-      <x:c r="C7" s="115"/>
-      <x:c r="D7" s="115"/>
-      <x:c r="E7" s="115" t="str">
+      <x:c r="D7" s="126"/>
+      <x:c r="E7" s="127" t="str">
+        <x:v>⚠️ 迷走</x:v>
+      </x:c>
+      <x:c r="F7" s="127"/>
+      <x:c r="G7" s="127" t="str">
         <x:v>0件 →</x:v>
       </x:c>
-      <x:c r="F7" s="115"/>
-      <x:c r="G7" s="115"/>
-      <x:c r="H7" s="115"/>
+      <x:c r="H7" s="127"/>
     </x:row>
     <x:row r="8" ht="18" customHeight="1">
-      <x:c r="A8" s="116" t="str">
+      <x:c r="A8" s="126" t="str">
         <x:v>📈 成長</x:v>
       </x:c>
-      <x:c r="B8" s="116"/>
-      <x:c r="C8" s="115"/>
-      <x:c r="D8" s="115"/>
-      <x:c r="E8" s="115" t="str">
-        <x:v>🌱 育成</x:v>
-      </x:c>
-      <x:c r="F8" s="115"/>
-      <x:c r="G8" s="115"/>
-      <x:c r="H8" s="115"/>
+      <x:c r="B8" s="126"/>
+      <x:c r="C8" s="126" t="str">
+        <x:v>0件 →</x:v>
+      </x:c>
+      <x:c r="D8" s="126"/>
+      <x:c r="E8" s="127" t="str">
+        <x:v>❓ 未取得</x:v>
+      </x:c>
+      <x:c r="F8" s="127"/>
+      <x:c r="G8" s="127" t="str">
+        <x:v>0件 →</x:v>
+      </x:c>
+      <x:c r="H8" s="127"/>
     </x:row>
     <x:row r="9" ht="18" customHeight="1">
-      <x:c r="A9" s="116" t="str">
-        <x:v>0件 →</x:v>
-      </x:c>
+      <x:c r="A9" s="116"/>
       <x:c r="B9" s="116"/>
       <x:c r="C9" s="115"/>
       <x:c r="D9" s="115"/>
-      <x:c r="E9" s="115" t="str">
-        <x:v>0件 →</x:v>
-      </x:c>
+      <x:c r="E9" s="115"/>
       <x:c r="F9" s="115"/>
       <x:c r="G9" s="115"/>
       <x:c r="H9" s="115"/>
     </x:row>
     <x:row r="10" ht="18" customHeight="1">
-      <x:c r="A10" s="116" t="str">
-        <x:v>⚠️ 低迷</x:v>
-      </x:c>
+      <x:c r="A10" s="116"/>
       <x:c r="B10" s="116"/>
       <x:c r="C10" s="115"/>
       <x:c r="D10" s="115"/>
-      <x:c r="E10" s="115" t="str">
-        <x:v>❓ 未取得</x:v>
-      </x:c>
+      <x:c r="E10" s="115"/>
       <x:c r="F10" s="115"/>
       <x:c r="G10" s="115"/>
       <x:c r="H10" s="115"/>
     </x:row>
     <x:row r="11" ht="18" customHeight="1">
-      <x:c r="A11" s="96" t="str">
-        <x:v>0件 →</x:v>
-      </x:c>
+      <x:c r="A11" s="96"/>
       <x:c r="B11" s="96"/>
       <x:c r="C11" s="96"/>
       <x:c r="D11" s="96"/>
-      <x:c r="E11" s="96" t="str">
-        <x:v>0件 →</x:v>
-      </x:c>
+      <x:c r="E11" s="96"/>
       <x:c r="F11" s="96"/>
       <x:c r="G11" s="96"/>
       <x:c r="H11" s="96"/>
     </x:row>
     <x:row r="12" ht="18" customHeight="1">
-      <x:c r="A12" s="118"/>
-      <x:c r="B12" s="118"/>
-      <x:c r="C12" s="118"/>
-      <x:c r="D12" s="118"/>
-      <x:c r="E12" s="118"/>
-      <x:c r="F12" s="118"/>
-      <x:c r="G12" s="118"/>
-      <x:c r="H12" s="118"/>
+      <x:c r="A12" s="96"/>
+      <x:c r="B12" s="96"/>
+      <x:c r="C12" s="96"/>
+      <x:c r="D12" s="96"/>
+      <x:c r="E12" s="96"/>
+      <x:c r="F12" s="96"/>
+      <x:c r="G12" s="96"/>
+      <x:c r="H12" s="96"/>
     </x:row>
     <x:row r="13" ht="18" customHeight="1">
-      <x:c r="A13" s="36" t="str">
+      <x:c r="A13" s="129" t="str">
         <x:v>改善状況</x:v>
       </x:c>
-      <x:c r="B13" s="36"/>
-      <x:c r="C13" s="36"/>
-      <x:c r="D13" s="36"/>
-      <x:c r="E13" s="36"/>
-      <x:c r="F13" s="36"/>
-      <x:c r="G13" s="36"/>
-      <x:c r="H13" s="36"/>
+      <x:c r="B13" s="129"/>
+      <x:c r="C13" s="129"/>
+      <x:c r="D13" s="129"/>
+      <x:c r="E13" s="129"/>
+      <x:c r="F13" s="129"/>
+      <x:c r="G13" s="129"/>
+      <x:c r="H13" s="129"/>
     </x:row>
     <x:row r="14" ht="18" customHeight="1">
       <x:c r="A14" s="88" t="str">
@@ -865,26 +933,26 @@
       <x:c r="H15" s="98"/>
     </x:row>
     <x:row r="16" ht="18" customHeight="1">
-      <x:c r="A16" s="120"/>
-      <x:c r="B16" s="120"/>
-      <x:c r="C16" s="120"/>
-      <x:c r="D16" s="120"/>
-      <x:c r="E16" s="120"/>
-      <x:c r="F16" s="120"/>
-      <x:c r="G16" s="120"/>
-      <x:c r="H16" s="120"/>
+      <x:c r="A16" s="98"/>
+      <x:c r="B16" s="98"/>
+      <x:c r="C16" s="98"/>
+      <x:c r="D16" s="98"/>
+      <x:c r="E16" s="98"/>
+      <x:c r="F16" s="98"/>
+      <x:c r="G16" s="98"/>
+      <x:c r="H16" s="98"/>
     </x:row>
     <x:row r="17" ht="18" customHeight="1">
-      <x:c r="A17" s="88" t="str">
+      <x:c r="A17" s="131" t="str">
         <x:v>今日のメッセージ</x:v>
       </x:c>
-      <x:c r="B17" s="88"/>
-      <x:c r="C17" s="36"/>
-      <x:c r="D17" s="36"/>
-      <x:c r="E17" s="36"/>
-      <x:c r="F17" s="36"/>
-      <x:c r="G17" s="36"/>
-      <x:c r="H17" s="36"/>
+      <x:c r="B17" s="131"/>
+      <x:c r="C17" s="131"/>
+      <x:c r="D17" s="131"/>
+      <x:c r="E17" s="131"/>
+      <x:c r="F17" s="131"/>
+      <x:c r="G17" s="131"/>
+      <x:c r="H17" s="131"/>
     </x:row>
     <x:row r="18" ht="18" customHeight="1">
       <x:c r="A18" s="88" t="str">
@@ -919,54 +987,54 @@
       <x:c r="H20" s="100"/>
     </x:row>
     <x:row r="21" ht="18" customHeight="1">
-      <x:c r="A21" s="122" t="str">
+      <x:c r="A21" s="132" t="str">
         <x:v>処理状況</x:v>
       </x:c>
-      <x:c r="B21" s="122"/>
-      <x:c r="C21" s="122"/>
-      <x:c r="D21" s="122"/>
-      <x:c r="E21" s="122"/>
-      <x:c r="F21" s="122"/>
-      <x:c r="G21" s="122"/>
-      <x:c r="H21" s="122"/>
+      <x:c r="B21" s="132"/>
+      <x:c r="C21" s="132"/>
+      <x:c r="D21" s="132"/>
+      <x:c r="E21" s="132"/>
+      <x:c r="F21" s="132"/>
+      <x:c r="G21" s="132"/>
+      <x:c r="H21" s="132"/>
     </x:row>
     <x:row r="22" ht="18" customHeight="1">
-      <x:c r="A22" s="121" t="str">
+      <x:c r="A22" s="133" t="str">
         <x:v>処理名</x:v>
       </x:c>
-      <x:c r="B22" s="121"/>
-      <x:c r="C22" s="121"/>
-      <x:c r="D22" s="121"/>
-      <x:c r="E22" s="121"/>
-      <x:c r="F22" s="121"/>
-      <x:c r="G22" s="121"/>
-      <x:c r="H22" s="121"/>
+      <x:c r="B22" s="133"/>
+      <x:c r="C22" s="133"/>
+      <x:c r="D22" s="133"/>
+      <x:c r="E22" s="133"/>
+      <x:c r="F22" s="133"/>
+      <x:c r="G22" s="133"/>
+      <x:c r="H22" s="133"/>
     </x:row>
     <x:row r="23" ht="18" customHeight="1">
-      <x:c r="A23" s="121" t="str">
+      <x:c r="A23" s="133" t="str">
         <x:v>開始時刻</x:v>
       </x:c>
-      <x:c r="B23" s="121"/>
-      <x:c r="C23" s="121"/>
-      <x:c r="D23" s="121" t="str">
+      <x:c r="B23" s="133"/>
+      <x:c r="C23" s="133"/>
+      <x:c r="D23" s="133" t="str">
         <x:v>処理結果</x:v>
       </x:c>
-      <x:c r="E23" s="121"/>
-      <x:c r="F23" s="121"/>
-      <x:c r="G23" s="121"/>
-      <x:c r="H23" s="121"/>
+      <x:c r="E23" s="133"/>
+      <x:c r="F23" s="133"/>
+      <x:c r="G23" s="133"/>
+      <x:c r="H23" s="133"/>
     </x:row>
     <x:row r="24" ht="18" customHeight="1">
-      <x:c r="A24" s="121" t="str">
+      <x:c r="A24" s="133" t="str">
         <x:v>お願い</x:v>
       </x:c>
-      <x:c r="B24" s="121"/>
-      <x:c r="C24" s="121"/>
-      <x:c r="D24" s="121"/>
-      <x:c r="E24" s="121"/>
-      <x:c r="F24" s="121"/>
-      <x:c r="G24" s="121"/>
-      <x:c r="H24" s="121"/>
+      <x:c r="B24" s="133"/>
+      <x:c r="C24" s="133"/>
+      <x:c r="D24" s="133"/>
+      <x:c r="E24" s="133"/>
+      <x:c r="F24" s="133"/>
+      <x:c r="G24" s="133"/>
+      <x:c r="H24" s="133"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="33"/>
@@ -1061,6 +1129,16 @@
     <x:mergeCell ref="B23:C23"/>
     <x:mergeCell ref="E23:H23"/>
     <x:mergeCell ref="B24:H24"/>
+    <x:mergeCell ref="C8:D8"/>
+    <x:mergeCell ref="E8:F8"/>
+    <x:mergeCell ref="G8:H8"/>
+    <x:mergeCell ref="A13:H13"/>
+    <x:mergeCell ref="A15:B15"/>
+    <x:mergeCell ref="C15:D15"/>
+    <x:mergeCell ref="E15:F15"/>
+    <x:mergeCell ref="G15:H15"/>
+    <x:mergeCell ref="A17:H17"/>
+    <x:mergeCell ref="A18:H19"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>